<commit_message>
Update raw datasets for Branchlet and Candlebark, and push latest boxplot
</commit_message>
<xml_diff>
--- a/Candlebark/candlebark.xlsx
+++ b/Candlebark/candlebark.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/Candle bark/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/Candlebark/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_A61340D536C40672D8AC891C568634196C229D73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3755BE2-6941-014D-9AB8-C1318EAFABE2}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="11_A61340D536C40672D8AC891C568634196C229D73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41457315-847E-AA4F-AEEA-F90EDD8367CF}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-5860" windowWidth="38400" windowHeight="21000" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-5860" windowWidth="38400" windowHeight="21000" firstSheet="4" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Curve 1 100 kW 60 cm_AUTO" sheetId="1" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4829" uniqueCount="1674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4829" uniqueCount="1670">
   <si>
     <t>Source.Name</t>
   </si>
@@ -4335,27 +4335,6 @@
     <t>0824_06_mesh.ply</t>
   </si>
   <si>
-    <t>0819_01_mesh_10.ply</t>
-  </si>
-  <si>
-    <t>0819_01_mesh_11.ply</t>
-  </si>
-  <si>
-    <t>0819_01_mesh_12.ply</t>
-  </si>
-  <si>
-    <t>0819_01_mesh_13.ply</t>
-  </si>
-  <si>
-    <t>0819_01_mesh_7.ply</t>
-  </si>
-  <si>
-    <t>0819_01_mesh_8.ply</t>
-  </si>
-  <si>
-    <t>0819_01_mesh_9.ply</t>
-  </si>
-  <si>
     <t>0819_04.csv</t>
   </si>
   <si>
@@ -5104,6 +5083,15 @@
   </si>
   <si>
     <t>Density (kg/m3)</t>
+  </si>
+  <si>
+    <t>0819_03_mesh_11.ply</t>
+  </si>
+  <si>
+    <t>0819_03_mesh_12.ply</t>
+  </si>
+  <si>
+    <t>0819_03_mesh_13.ply</t>
   </si>
 </sst>
 </file>
@@ -5156,10 +5144,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -16503,6 +16487,8 @@
   <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
     <col min="9" max="9" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16532,7 +16518,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>1673</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -16540,7 +16526,7 @@
         <v>756</v>
       </c>
       <c r="B2" t="s">
-        <v>743</v>
+        <v>757</v>
       </c>
       <c r="C2">
         <v>559.553</v>
@@ -16570,7 +16556,7 @@
         <v>756</v>
       </c>
       <c r="B3" t="s">
-        <v>1417</v>
+        <v>758</v>
       </c>
       <c r="C3">
         <v>654.92999999999995</v>
@@ -16600,7 +16586,7 @@
         <v>756</v>
       </c>
       <c r="B4" t="s">
-        <v>1418</v>
+        <v>1667</v>
       </c>
       <c r="C4">
         <v>750.30899999999997</v>
@@ -16630,7 +16616,7 @@
         <v>756</v>
       </c>
       <c r="B5" t="s">
-        <v>1419</v>
+        <v>1668</v>
       </c>
       <c r="C5">
         <v>437.31</v>
@@ -16660,7 +16646,7 @@
         <v>756</v>
       </c>
       <c r="B6" t="s">
-        <v>1420</v>
+        <v>1669</v>
       </c>
       <c r="C6">
         <v>230.66</v>
@@ -16690,7 +16676,7 @@
         <v>756</v>
       </c>
       <c r="B7" t="s">
-        <v>744</v>
+        <v>759</v>
       </c>
       <c r="C7">
         <v>448.84300000000002</v>
@@ -16720,7 +16706,7 @@
         <v>756</v>
       </c>
       <c r="B8" t="s">
-        <v>745</v>
+        <v>760</v>
       </c>
       <c r="C8">
         <v>908.80600000000004</v>
@@ -16750,7 +16736,7 @@
         <v>756</v>
       </c>
       <c r="B9" t="s">
-        <v>746</v>
+        <v>761</v>
       </c>
       <c r="C9">
         <v>326.60899999999998</v>
@@ -16780,7 +16766,7 @@
         <v>756</v>
       </c>
       <c r="B10" t="s">
-        <v>747</v>
+        <v>762</v>
       </c>
       <c r="C10">
         <v>437.572</v>
@@ -16810,7 +16796,7 @@
         <v>756</v>
       </c>
       <c r="B11" t="s">
-        <v>748</v>
+        <v>763</v>
       </c>
       <c r="C11">
         <v>190.78399999999999</v>
@@ -16840,7 +16826,7 @@
         <v>756</v>
       </c>
       <c r="B12" t="s">
-        <v>1421</v>
+        <v>764</v>
       </c>
       <c r="C12">
         <v>565.71699999999998</v>
@@ -16870,7 +16856,7 @@
         <v>756</v>
       </c>
       <c r="B13" t="s">
-        <v>1422</v>
+        <v>765</v>
       </c>
       <c r="C13">
         <v>587.14099999999996</v>
@@ -16900,7 +16886,7 @@
         <v>756</v>
       </c>
       <c r="B14" t="s">
-        <v>1423</v>
+        <v>766</v>
       </c>
       <c r="C14">
         <v>593.31100000000004</v>
@@ -16927,10 +16913,10 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B15" t="s">
-        <v>1425</v>
+        <v>1418</v>
       </c>
       <c r="C15">
         <v>251.07300000000001</v>
@@ -16957,10 +16943,10 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B16" t="s">
-        <v>1426</v>
+        <v>1419</v>
       </c>
       <c r="C16">
         <v>51.146999999999998</v>
@@ -16987,10 +16973,10 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B17" t="s">
-        <v>1427</v>
+        <v>1420</v>
       </c>
       <c r="C17">
         <v>39.796999999999997</v>
@@ -17017,10 +17003,10 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B18" t="s">
-        <v>1428</v>
+        <v>1421</v>
       </c>
       <c r="C18">
         <v>370.678</v>
@@ -17047,10 +17033,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B19" t="s">
-        <v>1429</v>
+        <v>1422</v>
       </c>
       <c r="C19">
         <v>111.804</v>
@@ -17077,10 +17063,10 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B20" t="s">
-        <v>1430</v>
+        <v>1423</v>
       </c>
       <c r="C20">
         <v>101.099</v>
@@ -17107,10 +17093,10 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>1417</v>
+      </c>
+      <c r="B21" t="s">
         <v>1424</v>
-      </c>
-      <c r="B21" t="s">
-        <v>1431</v>
       </c>
       <c r="C21">
         <v>209.06800000000001</v>
@@ -17137,10 +17123,10 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B22" t="s">
-        <v>1432</v>
+        <v>1425</v>
       </c>
       <c r="C22">
         <v>140.75399999999999</v>
@@ -17167,10 +17153,10 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B23" t="s">
-        <v>1433</v>
+        <v>1426</v>
       </c>
       <c r="C23">
         <v>55.308999999999997</v>
@@ -17197,10 +17183,10 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B24" t="s">
-        <v>1434</v>
+        <v>1427</v>
       </c>
       <c r="C24">
         <v>224.10499999999999</v>
@@ -17227,10 +17213,10 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B25" t="s">
-        <v>1435</v>
+        <v>1428</v>
       </c>
       <c r="C25">
         <v>198.95</v>
@@ -17257,10 +17243,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B26" t="s">
-        <v>1436</v>
+        <v>1429</v>
       </c>
       <c r="C26">
         <v>43.094999999999999</v>
@@ -17287,10 +17273,10 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B27" t="s">
-        <v>1437</v>
+        <v>1430</v>
       </c>
       <c r="C27">
         <v>102.97499999999999</v>
@@ -17317,10 +17303,10 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B28" t="s">
-        <v>1438</v>
+        <v>1431</v>
       </c>
       <c r="C28">
         <v>195.25700000000001</v>
@@ -17347,10 +17333,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B29" t="s">
-        <v>1439</v>
+        <v>1432</v>
       </c>
       <c r="C29">
         <v>75.295000000000002</v>
@@ -17377,10 +17363,10 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B30" t="s">
-        <v>1440</v>
+        <v>1433</v>
       </c>
       <c r="C30">
         <v>94.102000000000004</v>
@@ -17407,10 +17393,10 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B31" t="s">
-        <v>1441</v>
+        <v>1434</v>
       </c>
       <c r="C31">
         <v>90.918999999999997</v>
@@ -17437,10 +17423,10 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B32" t="s">
-        <v>1442</v>
+        <v>1435</v>
       </c>
       <c r="C32">
         <v>47.252000000000002</v>
@@ -17467,10 +17453,10 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B33" t="s">
-        <v>1443</v>
+        <v>1436</v>
       </c>
       <c r="C33">
         <v>92.444999999999993</v>
@@ -17497,10 +17483,10 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B34" t="s">
-        <v>1444</v>
+        <v>1437</v>
       </c>
       <c r="C34">
         <v>124.81100000000001</v>
@@ -17527,10 +17513,10 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B35" t="s">
-        <v>1445</v>
+        <v>1438</v>
       </c>
       <c r="C35">
         <v>64.221999999999994</v>
@@ -17827,7 +17813,7 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>1446</v>
+        <v>1439</v>
       </c>
       <c r="C12">
         <v>454.41699999999997</v>
@@ -17873,7 +17859,7 @@
         <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>1447</v>
+        <v>1440</v>
       </c>
       <c r="C14">
         <v>1128.5440000000001</v>
@@ -17896,7 +17882,7 @@
         <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>1448</v>
+        <v>1441</v>
       </c>
       <c r="C15">
         <v>785.64599999999996</v>
@@ -18758,10 +18744,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B2" t="s">
-        <v>1450</v>
+        <v>1443</v>
       </c>
       <c r="C2">
         <v>866.19399999999996</v>
@@ -18781,10 +18767,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B3" t="s">
-        <v>1451</v>
+        <v>1444</v>
       </c>
       <c r="C3">
         <v>266.76299999999998</v>
@@ -18804,10 +18790,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B4" t="s">
-        <v>1452</v>
+        <v>1445</v>
       </c>
       <c r="C4">
         <v>237.607</v>
@@ -18827,10 +18813,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B5" t="s">
-        <v>1453</v>
+        <v>1446</v>
       </c>
       <c r="C5">
         <v>644.60799999999995</v>
@@ -18850,10 +18836,10 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B6" t="s">
-        <v>1454</v>
+        <v>1447</v>
       </c>
       <c r="C6">
         <v>554.89800000000002</v>
@@ -18873,10 +18859,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B7" t="s">
-        <v>1455</v>
+        <v>1448</v>
       </c>
       <c r="C7">
         <v>926.96799999999996</v>
@@ -18896,10 +18882,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B8" t="s">
         <v>1449</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1456</v>
       </c>
       <c r="C8">
         <v>847.654</v>
@@ -18919,10 +18905,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B9" t="s">
-        <v>1457</v>
+        <v>1450</v>
       </c>
       <c r="C9">
         <v>215.56800000000001</v>
@@ -18942,10 +18928,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B10" t="s">
-        <v>1459</v>
+        <v>1452</v>
       </c>
       <c r="C10">
         <v>468.06</v>
@@ -18965,10 +18951,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B11" t="s">
-        <v>1460</v>
+        <v>1453</v>
       </c>
       <c r="C11">
         <v>336.709</v>
@@ -18988,10 +18974,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B12" t="s">
-        <v>1461</v>
+        <v>1454</v>
       </c>
       <c r="C12">
         <v>420.90600000000001</v>
@@ -19011,10 +18997,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B13" t="s">
-        <v>1462</v>
+        <v>1455</v>
       </c>
       <c r="C13">
         <v>28.027999999999999</v>
@@ -19034,10 +19020,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B14" t="s">
-        <v>1463</v>
+        <v>1456</v>
       </c>
       <c r="C14">
         <v>658.72699999999998</v>
@@ -19057,10 +19043,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B15" t="s">
-        <v>1464</v>
+        <v>1457</v>
       </c>
       <c r="C15">
         <v>14.053000000000001</v>
@@ -19080,10 +19066,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B16" t="s">
         <v>1458</v>
-      </c>
-      <c r="B16" t="s">
-        <v>1465</v>
       </c>
       <c r="C16">
         <v>218.898</v>
@@ -19103,10 +19089,10 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B17" t="s">
-        <v>1466</v>
+        <v>1459</v>
       </c>
       <c r="C17">
         <v>1184.7840000000001</v>
@@ -19126,10 +19112,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B18" t="s">
-        <v>1467</v>
+        <v>1460</v>
       </c>
       <c r="C18">
         <v>379.25700000000001</v>
@@ -19149,10 +19135,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B19" t="s">
-        <v>1468</v>
+        <v>1461</v>
       </c>
       <c r="C19">
         <v>147.13999999999999</v>
@@ -19172,10 +19158,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B20" t="s">
-        <v>1470</v>
+        <v>1463</v>
       </c>
       <c r="C20">
         <v>258.26</v>
@@ -19195,10 +19181,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B21" t="s">
-        <v>1471</v>
+        <v>1464</v>
       </c>
       <c r="C21">
         <v>265.358</v>
@@ -19218,10 +19204,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B22" t="s">
-        <v>1472</v>
+        <v>1465</v>
       </c>
       <c r="C22">
         <v>384.911</v>
@@ -19241,10 +19227,10 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B23" t="s">
-        <v>1473</v>
+        <v>1466</v>
       </c>
       <c r="C23">
         <v>1683.7909999999999</v>
@@ -19264,10 +19250,10 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B24" t="s">
-        <v>1474</v>
+        <v>1467</v>
       </c>
       <c r="C24">
         <v>104.699</v>
@@ -19287,10 +19273,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B25" t="s">
-        <v>1475</v>
+        <v>1468</v>
       </c>
       <c r="C25">
         <v>1086.8230000000001</v>
@@ -19310,10 +19296,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B26" t="s">
         <v>1469</v>
-      </c>
-      <c r="B26" t="s">
-        <v>1476</v>
       </c>
       <c r="C26">
         <v>265.524</v>
@@ -19333,10 +19319,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B27" t="s">
-        <v>1478</v>
+        <v>1471</v>
       </c>
       <c r="C27">
         <v>672.11500000000001</v>
@@ -19356,10 +19342,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B28" t="s">
-        <v>1479</v>
+        <v>1472</v>
       </c>
       <c r="C28">
         <v>645.39499999999998</v>
@@ -19379,10 +19365,10 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B29" t="s">
-        <v>1480</v>
+        <v>1473</v>
       </c>
       <c r="C29">
         <v>246.15700000000001</v>
@@ -19402,10 +19388,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B30" t="s">
-        <v>1481</v>
+        <v>1474</v>
       </c>
       <c r="C30">
         <v>75.820999999999998</v>
@@ -19425,10 +19411,10 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B31" t="s">
-        <v>1482</v>
+        <v>1475</v>
       </c>
       <c r="C31">
         <v>363.64100000000002</v>
@@ -19448,10 +19434,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B32" t="s">
-        <v>1483</v>
+        <v>1476</v>
       </c>
       <c r="C32">
         <v>139.44300000000001</v>
@@ -19471,10 +19457,10 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B33" t="s">
         <v>1477</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1484</v>
       </c>
       <c r="C33">
         <v>535.40300000000002</v>
@@ -19494,10 +19480,10 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B34" t="s">
-        <v>1485</v>
+        <v>1478</v>
       </c>
       <c r="C34">
         <v>501.113</v>
@@ -19517,10 +19503,10 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B35" t="s">
-        <v>1486</v>
+        <v>1479</v>
       </c>
       <c r="C35">
         <v>315.66699999999997</v>
@@ -19540,10 +19526,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B36" t="s">
-        <v>1487</v>
+        <v>1480</v>
       </c>
       <c r="C36">
         <v>32.648000000000003</v>
@@ -19563,10 +19549,10 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B37" t="s">
-        <v>1488</v>
+        <v>1481</v>
       </c>
       <c r="C37">
         <v>367.99099999999999</v>
@@ -19586,10 +19572,10 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B38" t="s">
-        <v>1489</v>
+        <v>1482</v>
       </c>
       <c r="C38">
         <v>182.95500000000001</v>
@@ -19609,10 +19595,10 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B39" t="s">
-        <v>1490</v>
+        <v>1483</v>
       </c>
       <c r="C39">
         <v>2017.865</v>
@@ -19632,10 +19618,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B40" t="s">
-        <v>1491</v>
+        <v>1484</v>
       </c>
       <c r="C40">
         <v>381.17200000000003</v>
@@ -19655,10 +19641,10 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B41" t="s">
-        <v>1493</v>
+        <v>1486</v>
       </c>
       <c r="C41">
         <v>455.23099999999999</v>
@@ -19678,10 +19664,10 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B42" t="s">
-        <v>1494</v>
+        <v>1487</v>
       </c>
       <c r="C42">
         <v>254.411</v>
@@ -19701,10 +19687,10 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B43" t="s">
-        <v>1495</v>
+        <v>1488</v>
       </c>
       <c r="C43">
         <v>76.155000000000001</v>
@@ -19724,10 +19710,10 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B44" t="s">
-        <v>1496</v>
+        <v>1489</v>
       </c>
       <c r="C44">
         <v>85.78</v>
@@ -19747,10 +19733,10 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B45" t="s">
-        <v>1497</v>
+        <v>1490</v>
       </c>
       <c r="C45">
         <v>144.155</v>
@@ -19770,10 +19756,10 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B46" t="s">
-        <v>1498</v>
+        <v>1491</v>
       </c>
       <c r="C46">
         <v>297.88600000000002</v>
@@ -19793,10 +19779,10 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
+        <v>1485</v>
+      </c>
+      <c r="B47" t="s">
         <v>1492</v>
-      </c>
-      <c r="B47" t="s">
-        <v>1499</v>
       </c>
       <c r="C47">
         <v>106.845</v>
@@ -19816,10 +19802,10 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B48" t="s">
-        <v>1500</v>
+        <v>1493</v>
       </c>
       <c r="C48">
         <v>358.10700000000003</v>
@@ -19839,10 +19825,10 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B49" t="s">
-        <v>1501</v>
+        <v>1494</v>
       </c>
       <c r="C49">
         <v>47.598999999999997</v>
@@ -19862,10 +19848,10 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B50" t="s">
-        <v>1502</v>
+        <v>1495</v>
       </c>
       <c r="C50">
         <v>370.21699999999998</v>
@@ -19885,10 +19871,10 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B51" t="s">
-        <v>1503</v>
+        <v>1496</v>
       </c>
       <c r="C51">
         <v>448.517</v>
@@ -19908,10 +19894,10 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B52" t="s">
-        <v>1504</v>
+        <v>1497</v>
       </c>
       <c r="C52">
         <v>409.51900000000001</v>
@@ -19931,10 +19917,10 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B53" t="s">
-        <v>1505</v>
+        <v>1498</v>
       </c>
       <c r="C53">
         <v>82.388000000000005</v>
@@ -19954,10 +19940,10 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B54" t="s">
-        <v>1506</v>
+        <v>1499</v>
       </c>
       <c r="C54">
         <v>227.63900000000001</v>
@@ -19977,10 +19963,10 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B55" t="s">
-        <v>1507</v>
+        <v>1500</v>
       </c>
       <c r="C55">
         <v>145.87299999999999</v>
@@ -20000,10 +19986,10 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B56" t="s">
-        <v>1508</v>
+        <v>1501</v>
       </c>
       <c r="C56">
         <v>553.30600000000004</v>
@@ -20023,10 +20009,10 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B57" t="s">
-        <v>1510</v>
+        <v>1503</v>
       </c>
       <c r="C57">
         <v>50.417999999999999</v>
@@ -20046,10 +20032,10 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B58" t="s">
-        <v>1511</v>
+        <v>1504</v>
       </c>
       <c r="C58">
         <v>136.19999999999999</v>
@@ -20069,10 +20055,10 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B59" t="s">
-        <v>1512</v>
+        <v>1505</v>
       </c>
       <c r="C59">
         <v>23.202000000000002</v>
@@ -20092,10 +20078,10 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B60" t="s">
-        <v>1513</v>
+        <v>1506</v>
       </c>
       <c r="C60">
         <v>142.48699999999999</v>
@@ -20115,10 +20101,10 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B61" t="s">
-        <v>1514</v>
+        <v>1507</v>
       </c>
       <c r="C61">
         <v>181.06800000000001</v>
@@ -20138,10 +20124,10 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B62" t="s">
-        <v>1515</v>
+        <v>1508</v>
       </c>
       <c r="C62">
         <v>1322.57</v>
@@ -20161,10 +20147,10 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B63" t="s">
         <v>1509</v>
-      </c>
-      <c r="B63" t="s">
-        <v>1516</v>
       </c>
       <c r="C63">
         <v>67.441000000000003</v>
@@ -20184,10 +20170,10 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B64" t="s">
-        <v>1517</v>
+        <v>1510</v>
       </c>
       <c r="C64">
         <v>164.22300000000001</v>
@@ -20207,10 +20193,10 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B65" t="s">
-        <v>1518</v>
+        <v>1511</v>
       </c>
       <c r="C65">
         <v>215.84</v>
@@ -20230,10 +20216,10 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B66" t="s">
-        <v>1519</v>
+        <v>1512</v>
       </c>
       <c r="C66">
         <v>760.71900000000005</v>
@@ -20253,10 +20239,10 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B67" t="s">
-        <v>1520</v>
+        <v>1513</v>
       </c>
       <c r="C67">
         <v>63.369</v>
@@ -20276,10 +20262,10 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B68" t="s">
-        <v>1521</v>
+        <v>1514</v>
       </c>
       <c r="C68">
         <v>84.424000000000007</v>
@@ -20299,10 +20285,10 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B69" t="s">
-        <v>1522</v>
+        <v>1515</v>
       </c>
       <c r="C69">
         <v>140.56399999999999</v>
@@ -20322,10 +20308,10 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B70" t="s">
-        <v>1523</v>
+        <v>1516</v>
       </c>
       <c r="C70">
         <v>50.981000000000002</v>
@@ -20345,10 +20331,10 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B71" t="s">
-        <v>1524</v>
+        <v>1517</v>
       </c>
       <c r="C71">
         <v>32.802</v>
@@ -20368,10 +20354,10 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B72" t="s">
-        <v>1525</v>
+        <v>1518</v>
       </c>
       <c r="C72">
         <v>69.91</v>
@@ -20391,10 +20377,10 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B73" t="s">
-        <v>1526</v>
+        <v>1519</v>
       </c>
       <c r="C73">
         <v>266.74400000000003</v>
@@ -20414,10 +20400,10 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B74" t="s">
-        <v>1527</v>
+        <v>1520</v>
       </c>
       <c r="C74">
         <v>117.491</v>
@@ -20437,10 +20423,10 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
       <c r="B75" t="s">
-        <v>1528</v>
+        <v>1521</v>
       </c>
       <c r="C75">
         <v>16.350999999999999</v>
@@ -20460,10 +20446,10 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>1529</v>
+        <v>1522</v>
       </c>
       <c r="B76" t="s">
-        <v>1530</v>
+        <v>1523</v>
       </c>
       <c r="C76">
         <v>5789.768</v>
@@ -20483,10 +20469,10 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>1529</v>
+        <v>1522</v>
       </c>
       <c r="B77" t="s">
-        <v>1531</v>
+        <v>1524</v>
       </c>
       <c r="C77">
         <v>3417.4850000000001</v>
@@ -20541,7 +20527,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>1673</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -21119,7 +21105,7 @@
         <v>370</v>
       </c>
       <c r="B21" t="s">
-        <v>1532</v>
+        <v>1525</v>
       </c>
       <c r="C21">
         <v>459.05</v>
@@ -23055,7 +23041,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>1446</v>
+        <v>1439</v>
       </c>
       <c r="C15">
         <v>433.55200000000002</v>
@@ -23078,7 +23064,7 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>1533</v>
+        <v>1526</v>
       </c>
       <c r="C16">
         <v>851.82</v>
@@ -24113,7 +24099,7 @@
         <v>355</v>
       </c>
       <c r="B61" t="s">
-        <v>1534</v>
+        <v>1527</v>
       </c>
       <c r="C61">
         <v>184.48400000000001</v>
@@ -24136,7 +24122,7 @@
         <v>355</v>
       </c>
       <c r="B62" t="s">
-        <v>1535</v>
+        <v>1528</v>
       </c>
       <c r="C62">
         <v>267.91000000000003</v>
@@ -24757,7 +24743,7 @@
         <v>370</v>
       </c>
       <c r="B89" t="s">
-        <v>1532</v>
+        <v>1525</v>
       </c>
       <c r="C89">
         <v>335.94400000000002</v>
@@ -24780,7 +24766,7 @@
         <v>370</v>
       </c>
       <c r="B90" t="s">
-        <v>1536</v>
+        <v>1529</v>
       </c>
       <c r="C90">
         <v>315.02</v>
@@ -24803,7 +24789,7 @@
         <v>370</v>
       </c>
       <c r="B91" t="s">
-        <v>1537</v>
+        <v>1530</v>
       </c>
       <c r="C91">
         <v>116.589</v>
@@ -24826,7 +24812,7 @@
         <v>370</v>
       </c>
       <c r="B92" t="s">
-        <v>1538</v>
+        <v>1531</v>
       </c>
       <c r="C92">
         <v>286.58699999999999</v>
@@ -24849,7 +24835,7 @@
         <v>370</v>
       </c>
       <c r="B93" t="s">
-        <v>1539</v>
+        <v>1532</v>
       </c>
       <c r="C93">
         <v>67.75</v>
@@ -24872,7 +24858,7 @@
         <v>370</v>
       </c>
       <c r="B94" t="s">
-        <v>1540</v>
+        <v>1533</v>
       </c>
       <c r="C94">
         <v>126.381</v>
@@ -24895,7 +24881,7 @@
         <v>370</v>
       </c>
       <c r="B95" t="s">
-        <v>1541</v>
+        <v>1534</v>
       </c>
       <c r="C95">
         <v>124.286</v>
@@ -24918,7 +24904,7 @@
         <v>370</v>
       </c>
       <c r="B96" t="s">
-        <v>1542</v>
+        <v>1535</v>
       </c>
       <c r="C96">
         <v>343.66699999999997</v>
@@ -25217,7 +25203,7 @@
         <v>380</v>
       </c>
       <c r="B109" t="s">
-        <v>1543</v>
+        <v>1536</v>
       </c>
       <c r="C109">
         <v>32.204999999999998</v>
@@ -25240,7 +25226,7 @@
         <v>380</v>
       </c>
       <c r="B110" t="s">
-        <v>1544</v>
+        <v>1537</v>
       </c>
       <c r="C110">
         <v>50.201000000000001</v>
@@ -25263,7 +25249,7 @@
         <v>380</v>
       </c>
       <c r="B111" t="s">
-        <v>1545</v>
+        <v>1538</v>
       </c>
       <c r="C111">
         <v>136.297</v>
@@ -25286,7 +25272,7 @@
         <v>380</v>
       </c>
       <c r="B112" t="s">
-        <v>1546</v>
+        <v>1539</v>
       </c>
       <c r="C112">
         <v>71.555999999999997</v>
@@ -25309,7 +25295,7 @@
         <v>380</v>
       </c>
       <c r="B113" t="s">
-        <v>1547</v>
+        <v>1540</v>
       </c>
       <c r="C113">
         <v>74.102999999999994</v>
@@ -25332,7 +25318,7 @@
         <v>380</v>
       </c>
       <c r="B114" t="s">
-        <v>1548</v>
+        <v>1541</v>
       </c>
       <c r="C114">
         <v>2.8420000000000001</v>
@@ -25355,7 +25341,7 @@
         <v>380</v>
       </c>
       <c r="B115" t="s">
-        <v>1549</v>
+        <v>1542</v>
       </c>
       <c r="C115">
         <v>66.177000000000007</v>
@@ -25401,7 +25387,7 @@
         <v>380</v>
       </c>
       <c r="B117" t="s">
-        <v>1550</v>
+        <v>1543</v>
       </c>
       <c r="C117">
         <v>82.92</v>
@@ -25424,7 +25410,7 @@
         <v>380</v>
       </c>
       <c r="B118" t="s">
-        <v>1551</v>
+        <v>1544</v>
       </c>
       <c r="C118">
         <v>72.031000000000006</v>
@@ -25447,7 +25433,7 @@
         <v>380</v>
       </c>
       <c r="B119" t="s">
-        <v>1552</v>
+        <v>1545</v>
       </c>
       <c r="C119">
         <v>108.117</v>
@@ -25470,7 +25456,7 @@
         <v>380</v>
       </c>
       <c r="B120" t="s">
-        <v>1553</v>
+        <v>1546</v>
       </c>
       <c r="C120">
         <v>84.105000000000004</v>
@@ -25493,7 +25479,7 @@
         <v>380</v>
       </c>
       <c r="B121" t="s">
-        <v>1554</v>
+        <v>1547</v>
       </c>
       <c r="C121">
         <v>42.853000000000002</v>
@@ -25516,7 +25502,7 @@
         <v>380</v>
       </c>
       <c r="B122" t="s">
-        <v>1555</v>
+        <v>1548</v>
       </c>
       <c r="C122">
         <v>85.355000000000004</v>
@@ -25732,7 +25718,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>1673</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -25830,7 +25816,7 @@
         <v>355</v>
       </c>
       <c r="B5" t="s">
-        <v>1534</v>
+        <v>1527</v>
       </c>
       <c r="C5">
         <v>257.49099999999999</v>
@@ -26307,10 +26293,10 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>1556</v>
+        <v>1549</v>
       </c>
       <c r="B21" t="s">
-        <v>1557</v>
+        <v>1550</v>
       </c>
       <c r="C21">
         <v>5224.5010000000002</v>
@@ -30751,10 +30737,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B14" t="s">
-        <v>1559</v>
+        <v>1552</v>
       </c>
       <c r="C14">
         <v>1421.21</v>
@@ -30774,10 +30760,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B15" t="s">
-        <v>1560</v>
+        <v>1553</v>
       </c>
       <c r="C15">
         <v>2009.6579999999999</v>
@@ -30797,10 +30783,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B16" t="s">
-        <v>1561</v>
+        <v>1554</v>
       </c>
       <c r="C16">
         <v>2220.1889999999999</v>
@@ -30820,10 +30806,10 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B17" t="s">
-        <v>1562</v>
+        <v>1555</v>
       </c>
       <c r="C17">
         <v>743.37900000000002</v>
@@ -30843,10 +30829,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B18" t="s">
-        <v>1563</v>
+        <v>1556</v>
       </c>
       <c r="C18">
         <v>13.657</v>
@@ -30866,10 +30852,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B19" t="s">
-        <v>1565</v>
+        <v>1558</v>
       </c>
       <c r="C19">
         <v>88.331999999999994</v>
@@ -30889,10 +30875,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B20" t="s">
-        <v>1566</v>
+        <v>1559</v>
       </c>
       <c r="C20">
         <v>35.139000000000003</v>
@@ -30912,10 +30898,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B21" t="s">
-        <v>1567</v>
+        <v>1560</v>
       </c>
       <c r="C21">
         <v>569.50199999999995</v>
@@ -30935,10 +30921,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B22" t="s">
-        <v>1568</v>
+        <v>1561</v>
       </c>
       <c r="C22">
         <v>1.236</v>
@@ -30958,10 +30944,10 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B23" t="s">
-        <v>1569</v>
+        <v>1562</v>
       </c>
       <c r="C23">
         <v>74.751999999999995</v>
@@ -30981,10 +30967,10 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B24" t="s">
-        <v>1570</v>
+        <v>1563</v>
       </c>
       <c r="C24">
         <v>801.63400000000001</v>
@@ -31004,10 +30990,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>1557</v>
+      </c>
+      <c r="B25" t="s">
         <v>1564</v>
-      </c>
-      <c r="B25" t="s">
-        <v>1571</v>
       </c>
       <c r="C25">
         <v>690.51400000000001</v>
@@ -31027,10 +31013,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B26" t="s">
-        <v>1572</v>
+        <v>1565</v>
       </c>
       <c r="C26">
         <v>417.178</v>
@@ -31050,10 +31036,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B27" t="s">
-        <v>1573</v>
+        <v>1566</v>
       </c>
       <c r="C27">
         <v>545.06899999999996</v>
@@ -31073,10 +31059,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B28" t="s">
-        <v>1574</v>
+        <v>1567</v>
       </c>
       <c r="C28">
         <v>263.99599999999998</v>
@@ -31096,10 +31082,10 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B29" t="s">
-        <v>1575</v>
+        <v>1568</v>
       </c>
       <c r="C29">
         <v>371.97</v>
@@ -31119,10 +31105,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B30" t="s">
-        <v>1576</v>
+        <v>1569</v>
       </c>
       <c r="C30">
         <v>362.05399999999997</v>
@@ -31142,10 +31128,10 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B31" t="s">
-        <v>1578</v>
+        <v>1571</v>
       </c>
       <c r="C31">
         <v>290.529</v>
@@ -31165,10 +31151,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B32" t="s">
-        <v>1579</v>
+        <v>1572</v>
       </c>
       <c r="C32">
         <v>278.08499999999998</v>
@@ -31188,10 +31174,10 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B33" t="s">
-        <v>1580</v>
+        <v>1573</v>
       </c>
       <c r="C33">
         <v>150.82</v>
@@ -31211,10 +31197,10 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B34" t="s">
-        <v>1581</v>
+        <v>1574</v>
       </c>
       <c r="C34">
         <v>631.23099999999999</v>
@@ -31234,10 +31220,10 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B35" t="s">
-        <v>1582</v>
+        <v>1575</v>
       </c>
       <c r="C35">
         <v>248.25200000000001</v>
@@ -31257,10 +31243,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B36" t="s">
-        <v>1583</v>
+        <v>1576</v>
       </c>
       <c r="C36">
         <v>325.83199999999999</v>
@@ -31280,10 +31266,10 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B37" t="s">
         <v>1577</v>
-      </c>
-      <c r="B37" t="s">
-        <v>1584</v>
       </c>
       <c r="C37">
         <v>74.072999999999993</v>
@@ -31303,10 +31289,10 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B38" t="s">
-        <v>1585</v>
+        <v>1578</v>
       </c>
       <c r="C38">
         <v>757.48400000000004</v>
@@ -31326,10 +31312,10 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B39" t="s">
-        <v>1586</v>
+        <v>1579</v>
       </c>
       <c r="C39">
         <v>288.625</v>
@@ -31349,10 +31335,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B40" t="s">
-        <v>1587</v>
+        <v>1580</v>
       </c>
       <c r="C40">
         <v>257.524</v>
@@ -31372,10 +31358,10 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B41" t="s">
-        <v>1588</v>
+        <v>1581</v>
       </c>
       <c r="C41">
         <v>268.43</v>
@@ -31395,10 +31381,10 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B42" t="s">
-        <v>1589</v>
+        <v>1582</v>
       </c>
       <c r="C42">
         <v>354.99</v>
@@ -31418,10 +31404,10 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B43" t="s">
-        <v>1590</v>
+        <v>1583</v>
       </c>
       <c r="C43">
         <v>233.80799999999999</v>
@@ -31441,10 +31427,10 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B44" t="s">
-        <v>1591</v>
+        <v>1584</v>
       </c>
       <c r="C44">
         <v>92.322000000000003</v>
@@ -31464,10 +31450,10 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B45" t="s">
-        <v>1592</v>
+        <v>1585</v>
       </c>
       <c r="C45">
         <v>83.331000000000003</v>
@@ -31487,10 +31473,10 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B46" t="s">
-        <v>1593</v>
+        <v>1586</v>
       </c>
       <c r="C46">
         <v>35.127000000000002</v>
@@ -31510,10 +31496,10 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
       <c r="B47" t="s">
-        <v>1594</v>
+        <v>1587</v>
       </c>
       <c r="C47">
         <v>102.017</v>
@@ -31533,10 +31519,10 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>1595</v>
+        <v>1588</v>
       </c>
       <c r="B48" t="s">
-        <v>1596</v>
+        <v>1589</v>
       </c>
       <c r="C48">
         <v>4871.723</v>
@@ -31556,10 +31542,10 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>1595</v>
+        <v>1588</v>
       </c>
       <c r="B49" t="s">
-        <v>1597</v>
+        <v>1590</v>
       </c>
       <c r="C49">
         <v>1605.2719999999999</v>
@@ -31616,10 +31602,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B2" t="s">
-        <v>1450</v>
+        <v>1443</v>
       </c>
       <c r="C2">
         <v>619.29899999999998</v>
@@ -31639,10 +31625,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B3" t="s">
-        <v>1451</v>
+        <v>1444</v>
       </c>
       <c r="C3">
         <v>1154.6199999999999</v>
@@ -31662,10 +31648,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B4" t="s">
-        <v>1452</v>
+        <v>1445</v>
       </c>
       <c r="C4">
         <v>478.49200000000002</v>
@@ -31685,10 +31671,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B5" t="s">
-        <v>1453</v>
+        <v>1446</v>
       </c>
       <c r="C5">
         <v>2060.962</v>
@@ -31708,10 +31694,10 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B6" t="s">
-        <v>1454</v>
+        <v>1447</v>
       </c>
       <c r="C6">
         <v>663.69200000000001</v>
@@ -31731,10 +31717,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B7" t="s">
-        <v>1455</v>
+        <v>1448</v>
       </c>
       <c r="C7">
         <v>253.89400000000001</v>
@@ -31754,10 +31740,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B8" t="s">
         <v>1449</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1456</v>
       </c>
       <c r="C8">
         <v>2149.3029999999999</v>
@@ -31777,10 +31763,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B9" t="s">
-        <v>1457</v>
+        <v>1450</v>
       </c>
       <c r="C9">
         <v>1.5469999999999999</v>
@@ -32056,7 +32042,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>1598</v>
+        <v>1591</v>
       </c>
       <c r="C21">
         <v>849.29399999999998</v>
@@ -32079,7 +32065,7 @@
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>1599</v>
+        <v>1592</v>
       </c>
       <c r="C22">
         <v>253.55199999999999</v>
@@ -32102,7 +32088,7 @@
         <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>1600</v>
+        <v>1593</v>
       </c>
       <c r="C23">
         <v>1254.6679999999999</v>
@@ -32125,7 +32111,7 @@
         <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>1601</v>
+        <v>1594</v>
       </c>
       <c r="C24">
         <v>880.54200000000003</v>
@@ -32263,7 +32249,7 @@
         <v>19</v>
       </c>
       <c r="B30" t="s">
-        <v>1446</v>
+        <v>1439</v>
       </c>
       <c r="C30">
         <v>293.404</v>
@@ -32286,7 +32272,7 @@
         <v>19</v>
       </c>
       <c r="B31" t="s">
-        <v>1533</v>
+        <v>1526</v>
       </c>
       <c r="C31">
         <v>53.433999999999997</v>
@@ -32309,7 +32295,7 @@
         <v>19</v>
       </c>
       <c r="B32" t="s">
-        <v>1602</v>
+        <v>1595</v>
       </c>
       <c r="C32">
         <v>308.55700000000002</v>
@@ -32355,7 +32341,7 @@
         <v>26</v>
       </c>
       <c r="B34" t="s">
-        <v>1447</v>
+        <v>1440</v>
       </c>
       <c r="C34">
         <v>339.46499999999997</v>
@@ -32378,7 +32364,7 @@
         <v>26</v>
       </c>
       <c r="B35" t="s">
-        <v>1448</v>
+        <v>1441</v>
       </c>
       <c r="C35">
         <v>241.95</v>
@@ -32401,7 +32387,7 @@
         <v>26</v>
       </c>
       <c r="B36" t="s">
-        <v>1603</v>
+        <v>1596</v>
       </c>
       <c r="C36">
         <v>401.286</v>
@@ -32424,7 +32410,7 @@
         <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>1604</v>
+        <v>1597</v>
       </c>
       <c r="C37">
         <v>997.67499999999995</v>
@@ -32447,7 +32433,7 @@
         <v>26</v>
       </c>
       <c r="B38" t="s">
-        <v>1605</v>
+        <v>1598</v>
       </c>
       <c r="C38">
         <v>105.919</v>
@@ -32470,7 +32456,7 @@
         <v>26</v>
       </c>
       <c r="B39" t="s">
-        <v>1606</v>
+        <v>1599</v>
       </c>
       <c r="C39">
         <v>119.29600000000001</v>
@@ -32493,7 +32479,7 @@
         <v>26</v>
       </c>
       <c r="B40" t="s">
-        <v>1607</v>
+        <v>1600</v>
       </c>
       <c r="C40">
         <v>299.89100000000002</v>
@@ -32516,7 +32502,7 @@
         <v>26</v>
       </c>
       <c r="B41" t="s">
-        <v>1608</v>
+        <v>1601</v>
       </c>
       <c r="C41">
         <v>98.376000000000005</v>
@@ -32539,7 +32525,7 @@
         <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>1609</v>
+        <v>1602</v>
       </c>
       <c r="C42">
         <v>108.175</v>
@@ -32562,7 +32548,7 @@
         <v>26</v>
       </c>
       <c r="B43" t="s">
-        <v>1610</v>
+        <v>1603</v>
       </c>
       <c r="C43">
         <v>643.22400000000005</v>
@@ -32608,7 +32594,7 @@
         <v>26</v>
       </c>
       <c r="B45" t="s">
-        <v>1611</v>
+        <v>1604</v>
       </c>
       <c r="C45">
         <v>153.20099999999999</v>
@@ -32861,7 +32847,7 @@
         <v>36</v>
       </c>
       <c r="B56" t="s">
-        <v>1612</v>
+        <v>1605</v>
       </c>
       <c r="C56">
         <v>62.786000000000001</v>
@@ -32884,7 +32870,7 @@
         <v>36</v>
       </c>
       <c r="B57" t="s">
-        <v>1613</v>
+        <v>1606</v>
       </c>
       <c r="C57">
         <v>397.75200000000001</v>
@@ -32907,7 +32893,7 @@
         <v>36</v>
       </c>
       <c r="B58" t="s">
-        <v>1614</v>
+        <v>1607</v>
       </c>
       <c r="C58">
         <v>0.56999999999999995</v>
@@ -32930,7 +32916,7 @@
         <v>36</v>
       </c>
       <c r="B59" t="s">
-        <v>1615</v>
+        <v>1608</v>
       </c>
       <c r="C59">
         <v>100.467</v>
@@ -32953,7 +32939,7 @@
         <v>36</v>
       </c>
       <c r="B60" t="s">
-        <v>1616</v>
+        <v>1609</v>
       </c>
       <c r="C60">
         <v>55.904000000000003</v>
@@ -32976,7 +32962,7 @@
         <v>36</v>
       </c>
       <c r="B61" t="s">
-        <v>1617</v>
+        <v>1610</v>
       </c>
       <c r="C61">
         <v>59.5</v>
@@ -32999,7 +32985,7 @@
         <v>36</v>
       </c>
       <c r="B62" t="s">
-        <v>1618</v>
+        <v>1611</v>
       </c>
       <c r="C62">
         <v>98.171999999999997</v>
@@ -33022,7 +33008,7 @@
         <v>36</v>
       </c>
       <c r="B63" t="s">
-        <v>1619</v>
+        <v>1612</v>
       </c>
       <c r="C63">
         <v>94.944999999999993</v>
@@ -33068,7 +33054,7 @@
         <v>36</v>
       </c>
       <c r="B65" t="s">
-        <v>1620</v>
+        <v>1613</v>
       </c>
       <c r="C65">
         <v>181.63300000000001</v>
@@ -33091,7 +33077,7 @@
         <v>36</v>
       </c>
       <c r="B66" t="s">
-        <v>1621</v>
+        <v>1614</v>
       </c>
       <c r="C66">
         <v>111.054</v>
@@ -33114,7 +33100,7 @@
         <v>36</v>
       </c>
       <c r="B67" t="s">
-        <v>1622</v>
+        <v>1615</v>
       </c>
       <c r="C67">
         <v>113.90300000000001</v>
@@ -33137,7 +33123,7 @@
         <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>1623</v>
+        <v>1616</v>
       </c>
       <c r="C68">
         <v>11.266999999999999</v>
@@ -33160,7 +33146,7 @@
         <v>36</v>
       </c>
       <c r="B69" t="s">
-        <v>1624</v>
+        <v>1617</v>
       </c>
       <c r="C69">
         <v>178.97200000000001</v>
@@ -33183,7 +33169,7 @@
         <v>36</v>
       </c>
       <c r="B70" t="s">
-        <v>1625</v>
+        <v>1618</v>
       </c>
       <c r="C70">
         <v>121.58499999999999</v>
@@ -33206,7 +33192,7 @@
         <v>36</v>
       </c>
       <c r="B71" t="s">
-        <v>1626</v>
+        <v>1619</v>
       </c>
       <c r="C71">
         <v>78.828000000000003</v>
@@ -33229,7 +33215,7 @@
         <v>36</v>
       </c>
       <c r="B72" t="s">
-        <v>1627</v>
+        <v>1620</v>
       </c>
       <c r="C72">
         <v>59.933</v>
@@ -33410,10 +33396,10 @@
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>1628</v>
+        <v>1621</v>
       </c>
       <c r="B80" t="s">
-        <v>1629</v>
+        <v>1622</v>
       </c>
       <c r="C80">
         <v>1207.7170000000001</v>
@@ -33433,10 +33419,10 @@
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>1628</v>
+        <v>1621</v>
       </c>
       <c r="B81" t="s">
-        <v>1630</v>
+        <v>1623</v>
       </c>
       <c r="C81">
         <v>2215.1320000000001</v>
@@ -33456,10 +33442,10 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>1628</v>
+        <v>1621</v>
       </c>
       <c r="B82" t="s">
-        <v>1631</v>
+        <v>1624</v>
       </c>
       <c r="C82">
         <v>1318.4860000000001</v>
@@ -33479,10 +33465,10 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>1628</v>
+        <v>1621</v>
       </c>
       <c r="B83" t="s">
-        <v>1632</v>
+        <v>1625</v>
       </c>
       <c r="C83">
         <v>4548.6409999999996</v>
@@ -33502,10 +33488,10 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>1628</v>
+        <v>1621</v>
       </c>
       <c r="B84" t="s">
-        <v>1633</v>
+        <v>1626</v>
       </c>
       <c r="C84">
         <v>5975.165</v>
@@ -33525,10 +33511,10 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>1628</v>
+        <v>1621</v>
       </c>
       <c r="B85" t="s">
-        <v>1634</v>
+        <v>1627</v>
       </c>
       <c r="C85">
         <v>6383.7960000000003</v>
@@ -33586,7 +33572,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>1673</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -33774,7 +33760,7 @@
         <v>749</v>
       </c>
       <c r="B8" t="s">
-        <v>1635</v>
+        <v>1628</v>
       </c>
       <c r="C8">
         <v>520.54300000000001</v>
@@ -33804,7 +33790,7 @@
         <v>749</v>
       </c>
       <c r="B9" t="s">
-        <v>1636</v>
+        <v>1629</v>
       </c>
       <c r="C9">
         <v>1023.772</v>
@@ -33834,7 +33820,7 @@
         <v>749</v>
       </c>
       <c r="B10" t="s">
-        <v>1637</v>
+        <v>1630</v>
       </c>
       <c r="C10">
         <v>37.314</v>
@@ -34014,7 +34000,7 @@
         <v>749</v>
       </c>
       <c r="B16" t="s">
-        <v>1638</v>
+        <v>1631</v>
       </c>
       <c r="C16">
         <v>690.33399999999995</v>
@@ -34044,7 +34030,7 @@
         <v>749</v>
       </c>
       <c r="B17" t="s">
-        <v>1639</v>
+        <v>1632</v>
       </c>
       <c r="C17">
         <v>122.712</v>
@@ -34074,7 +34060,7 @@
         <v>749</v>
       </c>
       <c r="B18" t="s">
-        <v>1640</v>
+        <v>1633</v>
       </c>
       <c r="C18">
         <v>910.71799999999996</v>
@@ -35417,10 +35403,10 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B17" t="s">
-        <v>1559</v>
+        <v>1552</v>
       </c>
       <c r="C17">
         <v>616.41800000000001</v>
@@ -35440,10 +35426,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B18" t="s">
-        <v>1560</v>
+        <v>1553</v>
       </c>
       <c r="C18">
         <v>1956.6389999999999</v>
@@ -35463,10 +35449,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B19" t="s">
-        <v>1561</v>
+        <v>1554</v>
       </c>
       <c r="C19">
         <v>3148.4810000000002</v>
@@ -35486,10 +35472,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B20" t="s">
-        <v>1562</v>
+        <v>1555</v>
       </c>
       <c r="C20">
         <v>1381.652</v>
@@ -35509,10 +35495,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B21" t="s">
-        <v>1563</v>
+        <v>1556</v>
       </c>
       <c r="C21">
         <v>1060.75</v>
@@ -35532,10 +35518,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B22" t="s">
-        <v>1641</v>
+        <v>1634</v>
       </c>
       <c r="C22">
         <v>484.08300000000003</v>
@@ -35555,10 +35541,10 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B23" t="s">
-        <v>1642</v>
+        <v>1635</v>
       </c>
       <c r="C23">
         <v>157.27600000000001</v>
@@ -35578,10 +35564,10 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
       <c r="B24" t="s">
-        <v>1643</v>
+        <v>1636</v>
       </c>
       <c r="C24">
         <v>968.447</v>
@@ -35601,10 +35587,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B25" t="s">
-        <v>1565</v>
+        <v>1558</v>
       </c>
       <c r="C25">
         <v>4000.009</v>
@@ -35624,10 +35610,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B26" t="s">
-        <v>1569</v>
+        <v>1562</v>
       </c>
       <c r="C26">
         <v>611.76099999999997</v>
@@ -35647,10 +35633,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B27" t="s">
-        <v>1570</v>
+        <v>1563</v>
       </c>
       <c r="C27">
         <v>549.55399999999997</v>
@@ -35670,10 +35656,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>1557</v>
+      </c>
+      <c r="B28" t="s">
         <v>1564</v>
-      </c>
-      <c r="B28" t="s">
-        <v>1571</v>
       </c>
       <c r="C28">
         <v>65.337000000000003</v>
@@ -35693,10 +35679,10 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B29" t="s">
-        <v>1572</v>
+        <v>1565</v>
       </c>
       <c r="C29">
         <v>963.46500000000003</v>
@@ -35716,10 +35702,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B30" t="s">
-        <v>1573</v>
+        <v>1566</v>
       </c>
       <c r="C30">
         <v>224.47800000000001</v>
@@ -35739,10 +35725,10 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B31" t="s">
-        <v>1574</v>
+        <v>1567</v>
       </c>
       <c r="C31">
         <v>1907.5260000000001</v>
@@ -35762,10 +35748,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B32" t="s">
-        <v>1575</v>
+        <v>1568</v>
       </c>
       <c r="C32">
         <v>332.928</v>
@@ -35785,10 +35771,10 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
       <c r="B33" t="s">
-        <v>1576</v>
+        <v>1569</v>
       </c>
       <c r="C33">
         <v>19.657</v>
@@ -35808,10 +35794,10 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B34" t="s">
-        <v>1450</v>
+        <v>1443</v>
       </c>
       <c r="C34">
         <v>486.899</v>
@@ -35831,10 +35817,10 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B35" t="s">
-        <v>1451</v>
+        <v>1444</v>
       </c>
       <c r="C35">
         <v>196.374</v>
@@ -35854,10 +35840,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B36" t="s">
-        <v>1452</v>
+        <v>1445</v>
       </c>
       <c r="C36">
         <v>1561.9390000000001</v>
@@ -35877,10 +35863,10 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B37" t="s">
-        <v>1453</v>
+        <v>1446</v>
       </c>
       <c r="C37">
         <v>3860.6170000000002</v>
@@ -35900,10 +35886,10 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B38" t="s">
-        <v>1454</v>
+        <v>1447</v>
       </c>
       <c r="C38">
         <v>527.01599999999996</v>
@@ -35923,10 +35909,10 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B39" t="s">
-        <v>1455</v>
+        <v>1448</v>
       </c>
       <c r="C39">
         <v>921.423</v>
@@ -35946,10 +35932,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B40" t="s">
         <v>1449</v>
-      </c>
-      <c r="B40" t="s">
-        <v>1456</v>
       </c>
       <c r="C40">
         <v>602.85299999999995</v>
@@ -35969,10 +35955,10 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B41" t="s">
-        <v>1457</v>
+        <v>1450</v>
       </c>
       <c r="C41">
         <v>516.27300000000002</v>
@@ -35992,10 +35978,10 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
       <c r="B42" t="s">
-        <v>1644</v>
+        <v>1637</v>
       </c>
       <c r="C42">
         <v>1056.3499999999999</v>
@@ -36015,10 +36001,10 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B43" t="s">
-        <v>1459</v>
+        <v>1452</v>
       </c>
       <c r="C43">
         <v>127.804</v>
@@ -36038,10 +36024,10 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B44" t="s">
-        <v>1460</v>
+        <v>1453</v>
       </c>
       <c r="C44">
         <v>203.899</v>
@@ -36061,10 +36047,10 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B45" t="s">
-        <v>1645</v>
+        <v>1638</v>
       </c>
       <c r="C45">
         <v>263.00099999999998</v>
@@ -36084,10 +36070,10 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B46" t="s">
-        <v>1646</v>
+        <v>1639</v>
       </c>
       <c r="C46">
         <v>186.94399999999999</v>
@@ -36107,10 +36093,10 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B47" t="s">
-        <v>1647</v>
+        <v>1640</v>
       </c>
       <c r="C47">
         <v>370.57799999999997</v>
@@ -36130,10 +36116,10 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B48" t="s">
-        <v>1648</v>
+        <v>1641</v>
       </c>
       <c r="C48">
         <v>482.52499999999998</v>
@@ -36153,10 +36139,10 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B49" t="s">
-        <v>1649</v>
+        <v>1642</v>
       </c>
       <c r="C49">
         <v>138.58500000000001</v>
@@ -36176,10 +36162,10 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B50" t="s">
-        <v>1650</v>
+        <v>1643</v>
       </c>
       <c r="C50">
         <v>314.82299999999998</v>
@@ -36199,10 +36185,10 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B51" t="s">
-        <v>1651</v>
+        <v>1644</v>
       </c>
       <c r="C51">
         <v>414.029</v>
@@ -36222,10 +36208,10 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B52" t="s">
-        <v>1461</v>
+        <v>1454</v>
       </c>
       <c r="C52">
         <v>13.737</v>
@@ -36245,10 +36231,10 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B53" t="s">
-        <v>1462</v>
+        <v>1455</v>
       </c>
       <c r="C53">
         <v>495.30099999999999</v>
@@ -36268,10 +36254,10 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B54" t="s">
-        <v>1463</v>
+        <v>1456</v>
       </c>
       <c r="C54">
         <v>332.84800000000001</v>
@@ -36291,10 +36277,10 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B55" t="s">
-        <v>1464</v>
+        <v>1457</v>
       </c>
       <c r="C55">
         <v>452.904</v>
@@ -36314,10 +36300,10 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B56" t="s">
         <v>1458</v>
-      </c>
-      <c r="B56" t="s">
-        <v>1465</v>
       </c>
       <c r="C56">
         <v>324.02100000000002</v>
@@ -36337,10 +36323,10 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B57" t="s">
-        <v>1466</v>
+        <v>1459</v>
       </c>
       <c r="C57">
         <v>164.06700000000001</v>
@@ -36360,10 +36346,10 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B58" t="s">
-        <v>1467</v>
+        <v>1460</v>
       </c>
       <c r="C58">
         <v>701.35599999999999</v>
@@ -36383,10 +36369,10 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
       <c r="B59" t="s">
-        <v>1468</v>
+        <v>1461</v>
       </c>
       <c r="C59">
         <v>1550.97</v>
@@ -36406,10 +36392,10 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B60" t="s">
-        <v>1470</v>
+        <v>1463</v>
       </c>
       <c r="C60">
         <v>178.27699999999999</v>
@@ -36429,10 +36415,10 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B61" t="s">
-        <v>1652</v>
+        <v>1645</v>
       </c>
       <c r="C61">
         <v>270.80700000000002</v>
@@ -36452,10 +36438,10 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B62" t="s">
-        <v>1653</v>
+        <v>1646</v>
       </c>
       <c r="C62">
         <v>178.26599999999999</v>
@@ -36475,10 +36461,10 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B63" t="s">
-        <v>1654</v>
+        <v>1647</v>
       </c>
       <c r="C63">
         <v>132.297</v>
@@ -36498,10 +36484,10 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B64" t="s">
-        <v>1655</v>
+        <v>1648</v>
       </c>
       <c r="C64">
         <v>317.298</v>
@@ -36521,10 +36507,10 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B65" t="s">
-        <v>1656</v>
+        <v>1649</v>
       </c>
       <c r="C65">
         <v>132.81700000000001</v>
@@ -36544,10 +36530,10 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B66" t="s">
-        <v>1657</v>
+        <v>1650</v>
       </c>
       <c r="C66">
         <v>100.709</v>
@@ -36567,10 +36553,10 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B67" t="s">
-        <v>1658</v>
+        <v>1651</v>
       </c>
       <c r="C67">
         <v>304.09899999999999</v>
@@ -36590,10 +36576,10 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B68" t="s">
-        <v>1659</v>
+        <v>1652</v>
       </c>
       <c r="C68">
         <v>136.73400000000001</v>
@@ -36613,10 +36599,10 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B69" t="s">
-        <v>1660</v>
+        <v>1653</v>
       </c>
       <c r="C69">
         <v>181.53399999999999</v>
@@ -36636,10 +36622,10 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B70" t="s">
-        <v>1661</v>
+        <v>1654</v>
       </c>
       <c r="C70">
         <v>229.86500000000001</v>
@@ -36659,10 +36645,10 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B71" t="s">
-        <v>1471</v>
+        <v>1464</v>
       </c>
       <c r="C71">
         <v>148.42500000000001</v>
@@ -36682,10 +36668,10 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B72" t="s">
-        <v>1662</v>
+        <v>1655</v>
       </c>
       <c r="C72">
         <v>252.73400000000001</v>
@@ -36705,10 +36691,10 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B73" t="s">
-        <v>1663</v>
+        <v>1656</v>
       </c>
       <c r="C73">
         <v>168.971</v>
@@ -36728,10 +36714,10 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B74" t="s">
-        <v>1664</v>
+        <v>1657</v>
       </c>
       <c r="C74">
         <v>178.64099999999999</v>
@@ -36751,10 +36737,10 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B75" t="s">
-        <v>1665</v>
+        <v>1658</v>
       </c>
       <c r="C75">
         <v>171.547</v>
@@ -36774,10 +36760,10 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B76" t="s">
-        <v>1472</v>
+        <v>1465</v>
       </c>
       <c r="C76">
         <v>203.31299999999999</v>
@@ -36797,10 +36783,10 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B77" t="s">
-        <v>1473</v>
+        <v>1466</v>
       </c>
       <c r="C77">
         <v>275.50900000000001</v>
@@ -36820,10 +36806,10 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B78" t="s">
-        <v>1474</v>
+        <v>1467</v>
       </c>
       <c r="C78">
         <v>155.06800000000001</v>
@@ -36843,10 +36829,10 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B79" t="s">
-        <v>1475</v>
+        <v>1468</v>
       </c>
       <c r="C79">
         <v>144.339</v>
@@ -36866,10 +36852,10 @@
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B80" t="s">
         <v>1469</v>
-      </c>
-      <c r="B80" t="s">
-        <v>1476</v>
       </c>
       <c r="C80">
         <v>212.14599999999999</v>
@@ -36889,10 +36875,10 @@
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B81" t="s">
-        <v>1666</v>
+        <v>1659</v>
       </c>
       <c r="C81">
         <v>91.15</v>
@@ -36912,10 +36898,10 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="B82" t="s">
-        <v>1667</v>
+        <v>1660</v>
       </c>
       <c r="C82">
         <v>330.40100000000001</v>
@@ -36935,10 +36921,10 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B83" t="s">
-        <v>1478</v>
+        <v>1471</v>
       </c>
       <c r="C83">
         <v>51.307000000000002</v>
@@ -36958,10 +36944,10 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B84" t="s">
-        <v>1479</v>
+        <v>1472</v>
       </c>
       <c r="C84">
         <v>127.10599999999999</v>
@@ -36981,10 +36967,10 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B85" t="s">
-        <v>1480</v>
+        <v>1473</v>
       </c>
       <c r="C85">
         <v>191.16399999999999</v>
@@ -37004,10 +36990,10 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B86" t="s">
-        <v>1481</v>
+        <v>1474</v>
       </c>
       <c r="C86">
         <v>93.989000000000004</v>
@@ -37027,10 +37013,10 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B87" t="s">
-        <v>1482</v>
+        <v>1475</v>
       </c>
       <c r="C87">
         <v>23.661000000000001</v>
@@ -37050,10 +37036,10 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B88" t="s">
-        <v>1483</v>
+        <v>1476</v>
       </c>
       <c r="C88">
         <v>82.619</v>
@@ -37073,10 +37059,10 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B89" t="s">
-        <v>1668</v>
+        <v>1661</v>
       </c>
       <c r="C89">
         <v>172.2</v>
@@ -37096,10 +37082,10 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B90" t="s">
         <v>1477</v>
-      </c>
-      <c r="B90" t="s">
-        <v>1484</v>
       </c>
       <c r="C90">
         <v>50.027999999999999</v>
@@ -37119,10 +37105,10 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B91" t="s">
-        <v>1485</v>
+        <v>1478</v>
       </c>
       <c r="C91">
         <v>172.79900000000001</v>
@@ -37142,10 +37128,10 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B92" t="s">
-        <v>1486</v>
+        <v>1479</v>
       </c>
       <c r="C92">
         <v>144.33500000000001</v>
@@ -37165,10 +37151,10 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B93" t="s">
-        <v>1487</v>
+        <v>1480</v>
       </c>
       <c r="C93">
         <v>138.83199999999999</v>
@@ -37188,10 +37174,10 @@
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B94" t="s">
-        <v>1488</v>
+        <v>1481</v>
       </c>
       <c r="C94">
         <v>119.407</v>
@@ -37211,10 +37197,10 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B95" t="s">
-        <v>1489</v>
+        <v>1482</v>
       </c>
       <c r="C95">
         <v>88.322000000000003</v>
@@ -37234,10 +37220,10 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B96" t="s">
-        <v>1490</v>
+        <v>1483</v>
       </c>
       <c r="C96">
         <v>41.548000000000002</v>
@@ -37257,10 +37243,10 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B97" t="s">
-        <v>1491</v>
+        <v>1484</v>
       </c>
       <c r="C97">
         <v>73.266999999999996</v>
@@ -37280,10 +37266,10 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>1669</v>
+        <v>1662</v>
       </c>
       <c r="B98" t="s">
-        <v>1670</v>
+        <v>1663</v>
       </c>
       <c r="C98">
         <v>4328.24</v>
@@ -37303,10 +37289,10 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>1669</v>
+        <v>1662</v>
       </c>
       <c r="B99" t="s">
-        <v>1671</v>
+        <v>1664</v>
       </c>
       <c r="C99">
         <v>1217.8050000000001</v>
@@ -37326,10 +37312,10 @@
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>1669</v>
+        <v>1662</v>
       </c>
       <c r="B100" t="s">
-        <v>1672</v>
+        <v>1665</v>
       </c>
       <c r="C100">
         <v>1652.6020000000001</v>
@@ -55086,7 +55072,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>1673</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update branchlet and candlebark raw data
</commit_message>
<xml_diff>
--- a/Candlebark/candlebark.xlsx
+++ b/Candlebark/candlebark.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/Candlebark/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="11_A61340D536C40672D8AC891C568634196C229D73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41457315-847E-AA4F-AEEA-F90EDD8367CF}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="11_A61340D536C40672D8AC891C568634196C229D73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80823F31-C40C-2841-B5E8-6E334932C30B}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-5860" windowWidth="38400" windowHeight="21000" firstSheet="4" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-5860" windowWidth="38400" windowHeight="21000" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Curve 1 100 kW 60 cm_AUTO" sheetId="1" r:id="rId1"/>
@@ -5144,6 +5144,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -55041,6 +55045,7 @@
   <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="2" max="2" width="28.1640625" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="16.83203125" customWidth="1"/>
@@ -55077,7 +55082,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="B2" t="s">
         <v>966</v>
@@ -55107,7 +55112,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="B3" t="s">
         <v>1220</v>
@@ -55167,7 +55172,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B5" t="s">
         <v>363</v>
@@ -55197,7 +55202,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B6" t="s">
         <v>1224</v>
@@ -55227,7 +55232,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B7" t="s">
         <v>1222</v>
@@ -55257,7 +55262,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B8" t="s">
         <v>1221</v>
@@ -55317,7 +55322,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="B10" t="s">
         <v>369</v>
@@ -55347,7 +55352,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B11" t="s">
         <v>969</v>
@@ -55467,7 +55472,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B15" t="s">
         <v>970</v>
@@ -55497,7 +55502,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="B16" t="s">
         <v>356</v>
@@ -55557,7 +55562,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="B18" t="s">
         <v>1226</v>
@@ -55587,7 +55592,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B19" t="s">
         <v>1229</v>
@@ -55617,7 +55622,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B20" t="s">
         <v>378</v>
@@ -55647,7 +55652,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B21" t="s">
         <v>968</v>
@@ -55767,7 +55772,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B25" t="s">
         <v>379</v>
@@ -55797,7 +55802,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B26" t="s">
         <v>967</v>
@@ -55827,7 +55832,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B27" t="s">
         <v>374</v>
@@ -55857,7 +55862,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="B28" t="s">
         <v>1217</v>
@@ -55917,7 +55922,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="B30" t="s">
         <v>373</v>
@@ -55947,7 +55952,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="B31" t="s">
         <v>1225</v>
@@ -56067,7 +56072,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B35" t="s">
         <v>377</v>
@@ -56097,7 +56102,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="B36" t="s">
         <v>359</v>
@@ -56157,7 +56162,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B38" t="s">
         <v>375</v>
@@ -56187,7 +56192,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B39" t="s">
         <v>376</v>
@@ -56217,7 +56222,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B40" t="s">
         <v>1230</v>
@@ -56247,7 +56252,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B41" t="s">
         <v>372</v>
@@ -56307,7 +56312,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="B43" t="s">
         <v>360</v>
@@ -56337,7 +56342,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="B44" t="s">
         <v>371</v>
@@ -56375,6 +56380,7 @@
     <sortCondition ref="I1:I44"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update Candlebark raw data and README
</commit_message>
<xml_diff>
--- a/Candlebark/candlebark.xlsx
+++ b/Candlebark/candlebark.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/Candlebark/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_A61340D536C40672D8AC891C568634196C229D73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80823F31-C40C-2841-B5E8-6E334932C30B}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="11_A61340D536C40672D8AC891C568634196C229D73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F927131-065C-1D43-B134-9CDEDCC78CC7}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-5860" windowWidth="38400" windowHeight="21000" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-5860" windowWidth="38400" windowHeight="21000" firstSheet="13" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Curve 1 100 kW 60 cm_AUTO" sheetId="1" r:id="rId1"/>
@@ -25695,6 +25695,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>